<commit_message>
v0.0.3 - mvp checked!)
</commit_message>
<xml_diff>
--- a/input/hyperlinksfile/1.xlsx
+++ b/input/hyperlinksfile/1.xlsx
@@ -24,56 +24,35 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="296">
   <si>
     <t>.2025             РОЗА</t>
   </si>
   <si>
-    <t>Роза ветвистая Викториан классик NL 60</t>
+    <t>BYN</t>
   </si>
   <si>
     <t>R Tr Victor Classic</t>
   </si>
   <si>
-    <t>Роза ветвистая Квинси NL 70</t>
-  </si>
-  <si>
     <t>R Tr Quincy</t>
   </si>
   <si>
-    <t>Роза ветвистая Лейла NL 70</t>
-  </si>
-  <si>
     <t>R Tr Leila</t>
   </si>
   <si>
-    <t>Роза ветвистая Пьяно красная NL 50</t>
-  </si>
-  <si>
     <t>R Tr Piano Freiland</t>
   </si>
   <si>
-    <t>Роза ветвистая Ред Трендсеттер NL 70</t>
-  </si>
-  <si>
     <t>R Tr Red Trendsetter</t>
   </si>
   <si>
-    <t>Роза ветвистая Резиденс NL 60</t>
-  </si>
-  <si>
     <t>R Tr Residence!</t>
   </si>
   <si>
-    <t>Роза ветвистая Сноуфлейк NL 50</t>
-  </si>
-  <si>
     <t>R Tr Snowflake</t>
   </si>
   <si>
-    <t>Роза ветвистая Сноуфлейк NL 60</t>
-  </si>
-  <si>
     <t>Хризантема 1 Антонов</t>
   </si>
   <si>
@@ -404,6 +383,9 @@
     <t>Aruncus Dioicus</t>
   </si>
   <si>
+    <t>Астильба розовая</t>
+  </si>
+  <si>
     <t>Astil Ja Europa</t>
   </si>
   <si>
@@ -911,7 +893,25 @@
     <t>Eus G Celeb Queen</t>
   </si>
   <si>
-    <t>роза арт деко</t>
+    <t>Роза ветвистая Пьяно красная NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Сноуфлейк NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Викториан классик NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Резиденс NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Квинси NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Лейла NL</t>
+  </si>
+  <si>
+    <t>Роза ветвистая Ред Трендсеттер NL</t>
   </si>
 </sst>
 </file>
@@ -1449,23 +1449,29 @@
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="2"/>
+      <c r="C1" s="2">
+        <v>2.95</v>
+      </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="7"/>
+        <v>291</v>
+      </c>
+      <c r="C3" s="7">
+        <v>9.74</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>2</v>
       </c>
@@ -1475,11 +1481,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C4" s="7">
+        <v>5.31</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="E4" s="8" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1487,11 +1495,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="7"/>
+        <v>294</v>
+      </c>
+      <c r="C5" s="7">
+        <v>5.31</v>
+      </c>
       <c r="E5" s="8" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1499,11 +1509,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="7"/>
+        <v>289</v>
+      </c>
+      <c r="C6" s="7">
+        <v>6.91</v>
+      </c>
       <c r="E6" s="8" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1511,11 +1523,13 @@
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="7"/>
+        <v>295</v>
+      </c>
+      <c r="C7" s="7">
+        <v>5.58</v>
+      </c>
       <c r="E7" s="8" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1523,11 +1537,13 @@
         <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="7"/>
+        <v>292</v>
+      </c>
+      <c r="C8" s="7">
+        <v>7.7799999999999994</v>
+      </c>
       <c r="E8" s="8" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1535,11 +1551,13 @@
         <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="7"/>
+        <v>290</v>
+      </c>
+      <c r="C9" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E9" s="8" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1547,11 +1565,13 @@
         <v>1</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="7"/>
+        <v>290</v>
+      </c>
+      <c r="C10" s="7">
+        <v>4.72</v>
+      </c>
       <c r="E10" s="8" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1559,11 +1579,13 @@
         <v>2</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="7"/>
+        <v>9</v>
+      </c>
+      <c r="C11" s="7">
+        <v>3.98</v>
+      </c>
       <c r="E11" s="8" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1571,11 +1593,13 @@
         <v>2</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="C12" s="7">
+        <v>4.41</v>
+      </c>
       <c r="E12" s="8" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1583,11 +1607,13 @@
         <v>2</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="9"/>
+        <v>13</v>
+      </c>
+      <c r="C13" s="9">
+        <v>4.25</v>
+      </c>
       <c r="E13" s="8" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1595,11 +1621,13 @@
         <v>2</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="C14" s="7">
+        <v>5.4399999999999995</v>
+      </c>
       <c r="E14" s="8" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1607,11 +1635,13 @@
         <v>2</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="9"/>
+        <v>17</v>
+      </c>
+      <c r="C15" s="9">
+        <v>4.25</v>
+      </c>
       <c r="E15" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1619,11 +1649,13 @@
         <v>2</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="9"/>
+        <v>19</v>
+      </c>
+      <c r="C16" s="9">
+        <v>3.69</v>
+      </c>
       <c r="E16" s="8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1631,11 +1663,13 @@
         <v>2</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="7"/>
+        <v>21</v>
+      </c>
+      <c r="C17" s="7">
+        <v>6.42</v>
+      </c>
       <c r="E17" s="8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1643,11 +1677,13 @@
         <v>2</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="9"/>
+        <v>23</v>
+      </c>
+      <c r="C18" s="9">
+        <v>5.76</v>
+      </c>
       <c r="E18" s="8" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1655,11 +1691,13 @@
         <v>2</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="7"/>
+        <v>25</v>
+      </c>
+      <c r="C19" s="7">
+        <v>5.22</v>
+      </c>
       <c r="E19" s="8" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1667,11 +1705,13 @@
         <v>2</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="C20" s="7">
+        <v>5.6099999999999994</v>
+      </c>
       <c r="E20" s="8" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1679,11 +1719,13 @@
         <v>2</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="7"/>
+        <v>29</v>
+      </c>
+      <c r="C21" s="7">
+        <v>4.2799999999999994</v>
+      </c>
       <c r="E21" s="8" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1691,11 +1733,13 @@
         <v>2</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="7"/>
+        <v>31</v>
+      </c>
+      <c r="C22" s="7">
+        <v>5.31</v>
+      </c>
       <c r="E22" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1703,11 +1747,13 @@
         <v>2</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="7"/>
+        <v>33</v>
+      </c>
+      <c r="C23" s="7">
+        <v>5.8199999999999994</v>
+      </c>
       <c r="E23" s="8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1715,11 +1761,13 @@
         <v>2</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="C24" s="7">
+        <v>4.13</v>
+      </c>
       <c r="E24" s="8" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1727,11 +1775,13 @@
         <v>2</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="7"/>
+        <v>37</v>
+      </c>
+      <c r="C25" s="7">
+        <v>5.39</v>
+      </c>
       <c r="E25" s="8" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1739,11 +1789,13 @@
         <v>2</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="C26" s="7">
+        <v>5.52</v>
+      </c>
       <c r="E26" s="8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1751,11 +1803,13 @@
         <v>2</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C27" s="7"/>
+        <v>41</v>
+      </c>
+      <c r="C27" s="7">
+        <v>4.92</v>
+      </c>
       <c r="E27" s="8" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1763,11 +1817,13 @@
         <v>2</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="7"/>
+        <v>43</v>
+      </c>
+      <c r="C28" s="7">
+        <v>4.58</v>
+      </c>
       <c r="E28" s="8" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1775,11 +1831,13 @@
         <v>2</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" s="7"/>
+        <v>45</v>
+      </c>
+      <c r="C29" s="7">
+        <v>4.58</v>
+      </c>
       <c r="E29" s="8" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1787,11 +1845,13 @@
         <v>2</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C30" s="7"/>
+        <v>47</v>
+      </c>
+      <c r="C30" s="7">
+        <v>5.31</v>
+      </c>
       <c r="E30" s="8" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1799,11 +1859,13 @@
         <v>2</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="7"/>
+        <v>49</v>
+      </c>
+      <c r="C31" s="7">
+        <v>5.52</v>
+      </c>
       <c r="E31" s="8" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1811,11 +1873,13 @@
         <v>2</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C32" s="7"/>
+        <v>51</v>
+      </c>
+      <c r="C32" s="7">
+        <v>4.58</v>
+      </c>
       <c r="E32" s="8" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1823,11 +1887,13 @@
         <v>2</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C33" s="7"/>
+        <v>53</v>
+      </c>
+      <c r="C33" s="7">
+        <v>3.4</v>
+      </c>
       <c r="E33" s="8" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1835,11 +1901,13 @@
         <v>2</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C34" s="7"/>
+        <v>55</v>
+      </c>
+      <c r="C34" s="7">
+        <v>6.79</v>
+      </c>
       <c r="E34" s="8" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1847,11 +1915,13 @@
         <v>2</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C35" s="7"/>
+        <v>57</v>
+      </c>
+      <c r="C35" s="7">
+        <v>5.6099999999999994</v>
+      </c>
       <c r="E35" s="8" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1859,11 +1929,13 @@
         <v>2</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C36" s="7"/>
+        <v>59</v>
+      </c>
+      <c r="C36" s="7">
+        <v>5.6099999999999994</v>
+      </c>
       <c r="E36" s="8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1871,11 +1943,13 @@
         <v>2</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C37" s="7"/>
+        <v>61</v>
+      </c>
+      <c r="C37" s="7">
+        <v>8.18</v>
+      </c>
       <c r="E37" s="8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1883,11 +1957,13 @@
         <v>2</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C38" s="7"/>
+        <v>63</v>
+      </c>
+      <c r="C38" s="7">
+        <v>5.22</v>
+      </c>
       <c r="E38" s="8" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1895,11 +1971,13 @@
         <v>2</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C39" s="7"/>
+        <v>65</v>
+      </c>
+      <c r="C39" s="7">
+        <v>4.58</v>
+      </c>
       <c r="E39" s="8" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1907,11 +1985,13 @@
         <v>2</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" s="7"/>
+        <v>67</v>
+      </c>
+      <c r="C40" s="7">
+        <v>2.95</v>
+      </c>
       <c r="E40" s="8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1919,11 +1999,13 @@
         <v>2</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C41" s="7"/>
+        <v>69</v>
+      </c>
+      <c r="C41" s="7">
+        <v>4.13</v>
+      </c>
       <c r="E41" s="8" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1931,11 +2013,13 @@
         <v>2</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" s="7"/>
+        <v>71</v>
+      </c>
+      <c r="C42" s="7">
+        <v>4.13</v>
+      </c>
       <c r="E42" s="8" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1943,11 +2027,13 @@
         <v>2</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C43" s="7"/>
+        <v>73</v>
+      </c>
+      <c r="C43" s="7">
+        <v>5.4399999999999995</v>
+      </c>
       <c r="E43" s="8" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1955,11 +2041,13 @@
         <v>2</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C44" s="7"/>
+        <v>75</v>
+      </c>
+      <c r="C44" s="7">
+        <v>5.4399999999999995</v>
+      </c>
       <c r="E44" s="8" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1967,11 +2055,13 @@
         <v>2</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C45" s="7"/>
+        <v>77</v>
+      </c>
+      <c r="C45" s="7">
+        <v>4.71</v>
+      </c>
       <c r="E45" s="8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1979,11 +2069,13 @@
         <v>2</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C46" s="7"/>
+        <v>79</v>
+      </c>
+      <c r="C46" s="7">
+        <v>3.4</v>
+      </c>
       <c r="E46" s="8" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1991,11 +2083,13 @@
         <v>2</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C47" s="7"/>
+        <v>81</v>
+      </c>
+      <c r="C47" s="7">
+        <v>3.84</v>
+      </c>
       <c r="E47" s="8" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2003,11 +2097,13 @@
         <v>4</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C48" s="7"/>
+        <v>83</v>
+      </c>
+      <c r="C48" s="7">
+        <v>64.900000000000006</v>
+      </c>
       <c r="E48" s="8" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2015,11 +2111,13 @@
         <v>4</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C49" s="7"/>
+        <v>85</v>
+      </c>
+      <c r="C49" s="7">
+        <v>70.8</v>
+      </c>
       <c r="E49" s="8" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2027,11 +2125,13 @@
         <v>4</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C50" s="7"/>
+        <v>87</v>
+      </c>
+      <c r="C50" s="7">
+        <v>64.900000000000006</v>
+      </c>
       <c r="E50" s="8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2039,11 +2139,13 @@
         <v>6</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C51" s="9"/>
+        <v>89</v>
+      </c>
+      <c r="C51" s="9">
+        <v>8.26</v>
+      </c>
       <c r="E51" s="8" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2051,11 +2153,13 @@
         <v>6</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C52" s="7"/>
+        <v>91</v>
+      </c>
+      <c r="C52" s="7">
+        <v>13.28</v>
+      </c>
       <c r="E52" s="8" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2063,11 +2167,13 @@
         <v>6</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C53" s="7"/>
+        <v>93</v>
+      </c>
+      <c r="C53" s="7">
+        <v>15.049999999999999</v>
+      </c>
       <c r="E53" s="8" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2075,11 +2181,13 @@
         <v>8</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C54" s="7"/>
+        <v>95</v>
+      </c>
+      <c r="C54" s="7">
+        <v>4.8999999999999995</v>
+      </c>
       <c r="E54" s="8" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2087,11 +2195,13 @@
         <v>8</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C55" s="7"/>
+        <v>97</v>
+      </c>
+      <c r="C55" s="7">
+        <v>3.54</v>
+      </c>
       <c r="E55" s="8" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2099,11 +2209,13 @@
         <v>8</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C56" s="7"/>
+        <v>99</v>
+      </c>
+      <c r="C56" s="7">
+        <v>3.54</v>
+      </c>
       <c r="E56" s="8" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2111,11 +2223,13 @@
         <v>8</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C57" s="7"/>
+        <v>101</v>
+      </c>
+      <c r="C57" s="7">
+        <v>19.71</v>
+      </c>
       <c r="E57" s="8" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2123,11 +2237,13 @@
         <v>8</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C58" s="7"/>
+        <v>103</v>
+      </c>
+      <c r="C58" s="7">
+        <v>5.81</v>
+      </c>
       <c r="E58" s="8" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2135,11 +2251,13 @@
         <v>8</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C59" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="C59" s="7">
+        <v>4.49</v>
+      </c>
       <c r="E59" s="8" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2147,11 +2265,13 @@
         <v>8</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C60" s="7"/>
+        <v>107</v>
+      </c>
+      <c r="C60" s="7">
+        <v>3.48</v>
+      </c>
       <c r="E60" s="8" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2159,11 +2279,13 @@
         <v>8</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C61" s="7"/>
+        <v>109</v>
+      </c>
+      <c r="C61" s="7">
+        <v>12.31</v>
+      </c>
       <c r="E61" s="8" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2171,11 +2293,13 @@
         <v>8</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C62" s="7"/>
+        <v>111</v>
+      </c>
+      <c r="C62" s="7">
+        <v>17.010000000000002</v>
+      </c>
       <c r="E62" s="8" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2183,11 +2307,13 @@
         <v>8</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C63" s="7"/>
+        <v>113</v>
+      </c>
+      <c r="C63" s="7">
+        <v>16.240000000000002</v>
+      </c>
       <c r="E63" s="8" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2195,11 +2321,13 @@
         <v>8</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C64" s="7"/>
+        <v>115</v>
+      </c>
+      <c r="C64" s="7">
+        <v>10.379999999999999</v>
+      </c>
       <c r="E64" s="8" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2207,11 +2335,13 @@
         <v>8</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="C65" s="7"/>
+        <v>117</v>
+      </c>
+      <c r="C65" s="7">
+        <v>3.3</v>
+      </c>
       <c r="E65" s="8" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2219,11 +2349,13 @@
         <v>8</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="C66" s="7"/>
+        <v>119</v>
+      </c>
+      <c r="C66" s="7">
+        <v>3.21</v>
+      </c>
       <c r="E66" s="8" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2231,11 +2363,13 @@
         <v>8</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C67" s="7"/>
+        <v>121</v>
+      </c>
+      <c r="C67" s="7">
+        <v>19.71</v>
+      </c>
       <c r="E67" s="8" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2243,11 +2377,13 @@
         <v>8</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="C68" s="7"/>
+        <v>123</v>
+      </c>
+      <c r="C68" s="7">
+        <v>6.13</v>
+      </c>
       <c r="E68" s="8" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2255,11 +2391,13 @@
         <v>8</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="C69" s="9"/>
+        <v>125</v>
+      </c>
+      <c r="C69" s="9">
+        <v>1.77</v>
+      </c>
       <c r="E69" s="8" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2267,11 +2405,13 @@
         <v>8</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="C70" s="9"/>
+        <v>127</v>
+      </c>
+      <c r="C70" s="9">
+        <v>1.77</v>
+      </c>
       <c r="E70" s="8" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2279,11 +2419,13 @@
         <v>8</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C71" s="7"/>
+        <v>129</v>
+      </c>
+      <c r="C71" s="7">
+        <v>2.5099999999999998</v>
+      </c>
       <c r="E71" s="8" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2291,11 +2433,13 @@
         <v>8</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="C72" s="7"/>
+        <v>131</v>
+      </c>
+      <c r="C72" s="7">
+        <v>2.5199999999999996</v>
+      </c>
       <c r="E72" s="8" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2303,11 +2447,13 @@
         <v>8</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C73" s="7"/>
+        <v>133</v>
+      </c>
+      <c r="C73" s="7">
+        <v>3.71</v>
+      </c>
       <c r="E73" s="8" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2315,11 +2461,13 @@
         <v>8</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="C74" s="7"/>
+        <v>135</v>
+      </c>
+      <c r="C74" s="7">
+        <v>2.5099999999999998</v>
+      </c>
       <c r="E74" s="8" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2327,11 +2475,13 @@
         <v>8</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C75" s="7"/>
+        <v>137</v>
+      </c>
+      <c r="C75" s="7">
+        <v>2.5099999999999998</v>
+      </c>
       <c r="E75" s="8" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2339,11 +2489,13 @@
         <v>8</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="C76" s="7"/>
+        <v>139</v>
+      </c>
+      <c r="C76" s="7">
+        <v>6.54</v>
+      </c>
       <c r="E76" s="8" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2351,11 +2503,13 @@
         <v>8</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C77" s="7"/>
+        <v>141</v>
+      </c>
+      <c r="C77" s="7">
+        <v>6.3199999999999994</v>
+      </c>
       <c r="E77" s="8" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2363,11 +2517,13 @@
         <v>8</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="C78" s="7"/>
+        <v>143</v>
+      </c>
+      <c r="C78" s="7">
+        <v>25.080000000000002</v>
+      </c>
       <c r="E78" s="8" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2375,11 +2531,13 @@
         <v>8</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="C79" s="7"/>
+        <v>145</v>
+      </c>
+      <c r="C79" s="7">
+        <v>26.55</v>
+      </c>
       <c r="E79" s="8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2387,11 +2545,13 @@
         <v>8</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="C80" s="7"/>
+        <v>147</v>
+      </c>
+      <c r="C80" s="7">
+        <v>19.180000000000003</v>
+      </c>
       <c r="E80" s="8" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2399,11 +2559,13 @@
         <v>8</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C81" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="C81" s="7">
+        <v>18.29</v>
+      </c>
       <c r="E81" s="8" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2411,11 +2573,13 @@
         <v>8</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C82" s="7"/>
+        <v>151</v>
+      </c>
+      <c r="C82" s="7">
+        <v>20.65</v>
+      </c>
       <c r="E82" s="8" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2423,11 +2587,13 @@
         <v>8</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C83" s="7"/>
+        <v>153</v>
+      </c>
+      <c r="C83" s="7">
+        <v>22.130000000000003</v>
+      </c>
       <c r="E83" s="8" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2435,11 +2601,13 @@
         <v>8</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="C84" s="7"/>
+        <v>155</v>
+      </c>
+      <c r="C84" s="7">
+        <v>16.23</v>
+      </c>
       <c r="E84" s="8" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2447,11 +2615,13 @@
         <v>8</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="C85" s="7"/>
+        <v>157</v>
+      </c>
+      <c r="C85" s="7">
+        <v>12.54</v>
+      </c>
       <c r="E85" s="8" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2459,11 +2629,13 @@
         <v>8</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="C86" s="7"/>
+        <v>159</v>
+      </c>
+      <c r="C86" s="7">
+        <v>12.54</v>
+      </c>
       <c r="E86" s="8" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2471,11 +2643,13 @@
         <v>8</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C87" s="7"/>
+        <v>161</v>
+      </c>
+      <c r="C87" s="7">
+        <v>2.2199999999999998</v>
+      </c>
       <c r="E87" s="8" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2483,11 +2657,13 @@
         <v>8</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="C88" s="7"/>
+        <v>163</v>
+      </c>
+      <c r="C88" s="7">
+        <v>2.2199999999999998</v>
+      </c>
       <c r="E88" s="8" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2495,11 +2671,13 @@
         <v>8</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C89" s="7"/>
+        <v>165</v>
+      </c>
+      <c r="C89" s="7">
+        <v>8.83</v>
+      </c>
       <c r="E89" s="8" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2507,11 +2685,13 @@
         <v>8</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="C90" s="7"/>
+        <v>167</v>
+      </c>
+      <c r="C90" s="7">
+        <v>14.129999999999999</v>
+      </c>
       <c r="E90" s="8" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2519,11 +2699,13 @@
         <v>8</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="C91" s="7"/>
+        <v>169</v>
+      </c>
+      <c r="C91" s="7">
+        <v>5.35</v>
+      </c>
       <c r="E91" s="8" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2531,11 +2713,13 @@
         <v>8</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C92" s="7"/>
+        <v>171</v>
+      </c>
+      <c r="C92" s="7">
+        <v>7.3199999999999994</v>
+      </c>
       <c r="E92" s="8" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2543,11 +2727,13 @@
         <v>8</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C93" s="7"/>
+        <v>173</v>
+      </c>
+      <c r="C93" s="7">
+        <v>4.26</v>
+      </c>
       <c r="E93" s="8" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2555,11 +2741,13 @@
         <v>8</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="C94" s="7"/>
+        <v>175</v>
+      </c>
+      <c r="C94" s="7">
+        <v>4.26</v>
+      </c>
       <c r="E94" s="8" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2567,11 +2755,13 @@
         <v>8</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C95" s="7"/>
+        <v>177</v>
+      </c>
+      <c r="C95" s="7">
+        <v>5.13</v>
+      </c>
       <c r="E95" s="8" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2579,11 +2769,13 @@
         <v>8</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="C96" s="7"/>
+        <v>179</v>
+      </c>
+      <c r="C96" s="7">
+        <v>2.95</v>
+      </c>
       <c r="E96" s="8" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2591,11 +2783,13 @@
         <v>8</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="C97" s="7"/>
+        <v>181</v>
+      </c>
+      <c r="C97" s="7">
+        <v>6.68</v>
+      </c>
       <c r="E97" s="8" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2603,11 +2797,13 @@
         <v>8</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="C98" s="7"/>
+        <v>183</v>
+      </c>
+      <c r="C98" s="7">
+        <v>5.17</v>
+      </c>
       <c r="E98" s="8" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2615,11 +2811,13 @@
         <v>8</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="C99" s="7"/>
+        <v>185</v>
+      </c>
+      <c r="C99" s="7">
+        <v>6.64</v>
+      </c>
       <c r="E99" s="8" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2627,11 +2825,13 @@
         <v>8</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C100" s="7"/>
+        <v>187</v>
+      </c>
+      <c r="C100" s="7">
+        <v>5.58</v>
+      </c>
       <c r="E100" s="8" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2639,11 +2839,13 @@
         <v>8</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C101" s="7"/>
+        <v>189</v>
+      </c>
+      <c r="C101" s="7">
+        <v>14.04</v>
+      </c>
       <c r="E101" s="8" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2651,11 +2853,13 @@
         <v>8</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="C102" s="7"/>
+        <v>191</v>
+      </c>
+      <c r="C102" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E102" s="8" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2663,11 +2867,13 @@
         <v>8</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="C103" s="7"/>
+        <v>193</v>
+      </c>
+      <c r="C103" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E103" s="8" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2675,11 +2881,13 @@
         <v>8</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="C104" s="7"/>
+        <v>195</v>
+      </c>
+      <c r="C104" s="7">
+        <v>4.87</v>
+      </c>
       <c r="E104" s="8" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2687,11 +2895,13 @@
         <v>8</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="C105" s="7"/>
+        <v>197</v>
+      </c>
+      <c r="C105" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E105" s="8" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2699,11 +2909,13 @@
         <v>8</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="C106" s="7"/>
+        <v>199</v>
+      </c>
+      <c r="C106" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E106" s="8" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2711,11 +2923,13 @@
         <v>8</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C107" s="7"/>
+        <v>201</v>
+      </c>
+      <c r="C107" s="7">
+        <v>4.43</v>
+      </c>
       <c r="E107" s="8" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2723,11 +2937,13 @@
         <v>8</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="C108" s="7"/>
+        <v>203</v>
+      </c>
+      <c r="C108" s="7">
+        <v>9.74</v>
+      </c>
       <c r="E108" s="8" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2735,11 +2951,13 @@
         <v>8</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="C109" s="7"/>
+        <v>205</v>
+      </c>
+      <c r="C109" s="7">
+        <v>2.95</v>
+      </c>
       <c r="E109" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2747,11 +2965,13 @@
         <v>8</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="C110" s="7"/>
+        <v>207</v>
+      </c>
+      <c r="C110" s="7">
+        <v>10.48</v>
+      </c>
       <c r="E110" s="8" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2759,11 +2979,13 @@
         <v>8</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C111" s="7"/>
+        <v>209</v>
+      </c>
+      <c r="C111" s="7">
+        <v>3.9899999999999998</v>
+      </c>
       <c r="E111" s="8" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2771,11 +2993,13 @@
         <v>8</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="C112" s="7"/>
+        <v>211</v>
+      </c>
+      <c r="C112" s="7">
+        <v>9.74</v>
+      </c>
       <c r="E112" s="8" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2783,11 +3007,13 @@
         <v>8</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="C113" s="7"/>
+        <v>213</v>
+      </c>
+      <c r="C113" s="7">
+        <v>9.74</v>
+      </c>
       <c r="E113" s="8" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2795,11 +3021,13 @@
         <v>8</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="C114" s="7"/>
+        <v>215</v>
+      </c>
+      <c r="C114" s="7">
+        <v>10.62</v>
+      </c>
       <c r="E114" s="8" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2807,11 +3035,13 @@
         <v>8</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="C115" s="7"/>
+        <v>217</v>
+      </c>
+      <c r="C115" s="7">
+        <v>10.34</v>
+      </c>
       <c r="E115" s="8" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2819,11 +3049,13 @@
         <v>8</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="C116" s="7"/>
+        <v>219</v>
+      </c>
+      <c r="C116" s="7">
+        <v>8.56</v>
+      </c>
       <c r="E116" s="8" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2831,11 +3063,13 @@
         <v>8</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="C117" s="7"/>
+        <v>221</v>
+      </c>
+      <c r="C117" s="7">
+        <v>10.18</v>
+      </c>
       <c r="E117" s="8" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="118" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2843,11 +3077,13 @@
         <v>8</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="C118" s="7"/>
+        <v>223</v>
+      </c>
+      <c r="C118" s="7">
+        <v>8.26</v>
+      </c>
       <c r="E118" s="8" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="119" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2855,11 +3091,13 @@
         <v>8</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="C119" s="7"/>
+        <v>225</v>
+      </c>
+      <c r="C119" s="7">
+        <v>21.680000000000003</v>
+      </c>
       <c r="E119" s="8" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="120" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2867,11 +3105,13 @@
         <v>8</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="C120" s="7"/>
+        <v>227</v>
+      </c>
+      <c r="C120" s="7">
+        <v>54.919999999999995</v>
+      </c>
       <c r="E120" s="8" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="121" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2879,11 +3119,13 @@
         <v>8</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="C121" s="7"/>
+        <v>229</v>
+      </c>
+      <c r="C121" s="7">
+        <v>25.430000000000003</v>
+      </c>
       <c r="E121" s="8" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="122" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2891,11 +3133,13 @@
         <v>8</v>
       </c>
       <c r="B122" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="C122" s="7"/>
+        <v>231</v>
+      </c>
+      <c r="C122" s="7">
+        <v>14.18</v>
+      </c>
       <c r="E122" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2903,11 +3147,13 @@
         <v>8</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="C123" s="7"/>
+        <v>233</v>
+      </c>
+      <c r="C123" s="7">
+        <v>4.3899999999999997</v>
+      </c>
       <c r="E123" s="8" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2915,11 +3161,13 @@
         <v>8</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="C124" s="7"/>
+        <v>235</v>
+      </c>
+      <c r="C124" s="7">
+        <v>3.9899999999999998</v>
+      </c>
       <c r="E124" s="8" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="125" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2927,11 +3175,13 @@
         <v>8</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="C125" s="7"/>
+        <v>237</v>
+      </c>
+      <c r="C125" s="7">
+        <v>3.9899999999999998</v>
+      </c>
       <c r="E125" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="126" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2939,11 +3189,13 @@
         <v>8</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="C126" s="7"/>
+        <v>239</v>
+      </c>
+      <c r="C126" s="7">
+        <v>3.9899999999999998</v>
+      </c>
       <c r="E126" s="8" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="127" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2951,11 +3203,13 @@
         <v>8</v>
       </c>
       <c r="B127" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="C127" s="7"/>
+        <v>241</v>
+      </c>
+      <c r="C127" s="7">
+        <v>13.86</v>
+      </c>
       <c r="E127" s="8" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2963,11 +3217,13 @@
         <v>8</v>
       </c>
       <c r="B128" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="C128" s="7"/>
+        <v>243</v>
+      </c>
+      <c r="C128" s="7">
+        <v>4.72</v>
+      </c>
       <c r="E128" s="8" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="129" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2975,11 +3231,13 @@
         <v>8</v>
       </c>
       <c r="B129" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="C129" s="7"/>
+        <v>245</v>
+      </c>
+      <c r="C129" s="7">
+        <v>5.31</v>
+      </c>
       <c r="E129" s="8" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2987,11 +3245,13 @@
         <v>8</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="C130" s="9"/>
+        <v>247</v>
+      </c>
+      <c r="C130" s="9">
+        <v>2.0699999999999998</v>
+      </c>
       <c r="E130" s="8" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="131" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2999,11 +3259,13 @@
         <v>8</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="C131" s="7"/>
+        <v>249</v>
+      </c>
+      <c r="C131" s="7">
+        <v>8.3699999999999992</v>
+      </c>
       <c r="E131" s="8" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="132" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3011,11 +3273,13 @@
         <v>8</v>
       </c>
       <c r="B132" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="C132" s="7"/>
+        <v>251</v>
+      </c>
+      <c r="C132" s="7">
+        <v>6.54</v>
+      </c>
       <c r="E132" s="8" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="133" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3023,11 +3287,13 @@
         <v>8</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="C133" s="7"/>
+        <v>253</v>
+      </c>
+      <c r="C133" s="7">
+        <v>3.54</v>
+      </c>
       <c r="E133" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="134" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3035,11 +3301,13 @@
         <v>8</v>
       </c>
       <c r="B134" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="C134" s="9"/>
+        <v>255</v>
+      </c>
+      <c r="C134" s="9">
+        <v>2.95</v>
+      </c>
       <c r="E134" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="135" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3047,11 +3315,13 @@
         <v>8</v>
       </c>
       <c r="B135" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="C135" s="9"/>
+        <v>257</v>
+      </c>
+      <c r="C135" s="9">
+        <v>3.25</v>
+      </c>
       <c r="E135" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
     </row>
     <row r="136" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3059,11 +3329,13 @@
         <v>8</v>
       </c>
       <c r="B136" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="C136" s="9"/>
+        <v>259</v>
+      </c>
+      <c r="C136" s="9">
+        <v>6.2</v>
+      </c>
       <c r="E136" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3071,11 +3343,13 @@
         <v>8</v>
       </c>
       <c r="B137" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="C137" s="7"/>
+        <v>261</v>
+      </c>
+      <c r="C137" s="7">
+        <v>10.029999999999999</v>
+      </c>
       <c r="E137" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="138" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3083,11 +3357,13 @@
         <v>8</v>
       </c>
       <c r="B138" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="C138" s="7"/>
+        <v>262</v>
+      </c>
+      <c r="C138" s="7">
+        <v>8.26</v>
+      </c>
       <c r="E138" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="139" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3095,11 +3371,13 @@
         <v>8</v>
       </c>
       <c r="B139" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="C139" s="7"/>
+        <v>264</v>
+      </c>
+      <c r="C139" s="7">
+        <v>10.029999999999999</v>
+      </c>
       <c r="E139" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="140" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3107,11 +3385,13 @@
         <v>8</v>
       </c>
       <c r="B140" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="C140" s="7"/>
+        <v>265</v>
+      </c>
+      <c r="C140" s="7">
+        <v>8.26</v>
+      </c>
       <c r="E140" s="8" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
     </row>
     <row r="141" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3119,11 +3399,13 @@
         <v>8</v>
       </c>
       <c r="B141" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="C141" s="7"/>
+        <v>267</v>
+      </c>
+      <c r="C141" s="7">
+        <v>10.029999999999999</v>
+      </c>
       <c r="E141" s="8" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3131,11 +3413,13 @@
         <v>8</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="C142" s="9"/>
+        <v>269</v>
+      </c>
+      <c r="C142" s="9">
+        <v>4.87</v>
+      </c>
       <c r="E142" s="8" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3143,11 +3427,13 @@
         <v>8</v>
       </c>
       <c r="B143" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="C143" s="9"/>
+        <v>271</v>
+      </c>
+      <c r="C143" s="9">
+        <v>5.9</v>
+      </c>
       <c r="E143" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
     </row>
     <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3155,11 +3441,13 @@
         <v>8</v>
       </c>
       <c r="B144" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="C144" s="9"/>
+        <v>273</v>
+      </c>
+      <c r="C144" s="9">
+        <v>5.9</v>
+      </c>
       <c r="E144" s="8" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
     </row>
     <row r="145" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3167,11 +3455,13 @@
         <v>8</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="C145" s="7"/>
+        <v>275</v>
+      </c>
+      <c r="C145" s="7">
+        <v>11.21</v>
+      </c>
       <c r="E145" s="8" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
     </row>
     <row r="146" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3179,11 +3469,13 @@
         <v>8</v>
       </c>
       <c r="B146" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="C146" s="7"/>
+        <v>277</v>
+      </c>
+      <c r="C146" s="7">
+        <v>8.85</v>
+      </c>
       <c r="E146" s="8" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
     </row>
     <row r="147" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3191,11 +3483,13 @@
         <v>8</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="C147" s="7"/>
+        <v>279</v>
+      </c>
+      <c r="C147" s="7">
+        <v>6.49</v>
+      </c>
       <c r="E147" s="8" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
     </row>
     <row r="148" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3203,11 +3497,13 @@
         <v>8</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="C148" s="7"/>
+        <v>281</v>
+      </c>
+      <c r="C148" s="7">
+        <v>7.38</v>
+      </c>
       <c r="E148" s="8" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="149" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3215,11 +3511,13 @@
         <v>8</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="C149" s="7"/>
+        <v>283</v>
+      </c>
+      <c r="C149" s="7">
+        <v>7.96</v>
+      </c>
       <c r="E149" s="8" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="150" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3227,11 +3525,13 @@
         <v>8</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="C150" s="7"/>
+        <v>285</v>
+      </c>
+      <c r="C150" s="7">
+        <v>10.33</v>
+      </c>
       <c r="E150" s="8" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
     </row>
     <row r="151" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3239,11 +3539,13 @@
         <v>8</v>
       </c>
       <c r="B151" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="C151" s="7"/>
+        <v>287</v>
+      </c>
+      <c r="C151" s="7">
+        <v>11.21</v>
+      </c>
       <c r="E151" s="8" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
     </row>
     <row r="152" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3253,7 +3555,9 @@
       <c r="B152" s="6">
         <v>0</v>
       </c>
-      <c r="C152" s="7"/>
+      <c r="C152" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E152">
         <v>0</v>
       </c>
@@ -3265,7 +3569,9 @@
       <c r="B153" s="6">
         <v>0</v>
       </c>
-      <c r="C153" s="7"/>
+      <c r="C153" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E153">
         <v>0</v>
       </c>
@@ -3277,7 +3583,9 @@
       <c r="B154" s="6">
         <v>0</v>
       </c>
-      <c r="C154" s="7"/>
+      <c r="C154" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E154">
         <v>0</v>
       </c>
@@ -3289,7 +3597,9 @@
       <c r="B155" s="6">
         <v>0</v>
       </c>
-      <c r="C155" s="7"/>
+      <c r="C155" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E155">
         <v>0</v>
       </c>
@@ -3301,7 +3611,9 @@
       <c r="B156" s="6">
         <v>0</v>
       </c>
-      <c r="C156" s="7"/>
+      <c r="C156" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E156">
         <v>0</v>
       </c>
@@ -3313,7 +3625,9 @@
       <c r="B157" s="6">
         <v>0</v>
       </c>
-      <c r="C157" s="7"/>
+      <c r="C157" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E157">
         <v>0</v>
       </c>
@@ -3325,7 +3639,9 @@
       <c r="B158" s="6">
         <v>0</v>
       </c>
-      <c r="C158" s="7"/>
+      <c r="C158" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E158">
         <v>0</v>
       </c>
@@ -3337,7 +3653,9 @@
       <c r="B159" s="6">
         <v>0</v>
       </c>
-      <c r="C159" s="7"/>
+      <c r="C159" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E159">
         <v>0</v>
       </c>
@@ -3349,7 +3667,9 @@
       <c r="B160" s="6">
         <v>0</v>
       </c>
-      <c r="C160" s="7"/>
+      <c r="C160" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E160">
         <v>0</v>
       </c>
@@ -3361,7 +3681,9 @@
       <c r="B161" s="6">
         <v>0</v>
       </c>
-      <c r="C161" s="7"/>
+      <c r="C161" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E161">
         <v>0</v>
       </c>
@@ -3373,7 +3695,9 @@
       <c r="B162" s="6">
         <v>0</v>
       </c>
-      <c r="C162" s="7"/>
+      <c r="C162" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E162">
         <v>0</v>
       </c>
@@ -3385,7 +3709,9 @@
       <c r="B163" s="6">
         <v>0</v>
       </c>
-      <c r="C163" s="7"/>
+      <c r="C163" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E163">
         <v>0</v>
       </c>
@@ -3397,7 +3723,9 @@
       <c r="B164" s="6">
         <v>0</v>
       </c>
-      <c r="C164" s="7"/>
+      <c r="C164" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E164">
         <v>0</v>
       </c>
@@ -3409,7 +3737,9 @@
       <c r="B165" s="6">
         <v>0</v>
       </c>
-      <c r="C165" s="7"/>
+      <c r="C165" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E165">
         <v>0</v>
       </c>
@@ -3421,7 +3751,9 @@
       <c r="B166" s="6">
         <v>0</v>
       </c>
-      <c r="C166" s="7"/>
+      <c r="C166" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E166">
         <v>0</v>
       </c>
@@ -3433,7 +3765,9 @@
       <c r="B167" s="6">
         <v>0</v>
       </c>
-      <c r="C167" s="7"/>
+      <c r="C167" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E167">
         <v>0</v>
       </c>
@@ -3445,7 +3779,9 @@
       <c r="B168" s="6">
         <v>0</v>
       </c>
-      <c r="C168" s="7"/>
+      <c r="C168" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E168">
         <v>0</v>
       </c>
@@ -3457,7 +3793,9 @@
       <c r="B169" s="6">
         <v>0</v>
       </c>
-      <c r="C169" s="7"/>
+      <c r="C169" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E169">
         <v>0</v>
       </c>
@@ -3469,7 +3807,9 @@
       <c r="B170" s="6">
         <v>0</v>
       </c>
-      <c r="C170" s="7"/>
+      <c r="C170" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E170">
         <v>0</v>
       </c>
@@ -3481,7 +3821,9 @@
       <c r="B171" s="6">
         <v>0</v>
       </c>
-      <c r="C171" s="7"/>
+      <c r="C171" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E171">
         <v>0</v>
       </c>
@@ -3493,7 +3835,9 @@
       <c r="B172" s="6">
         <v>0</v>
       </c>
-      <c r="C172" s="7"/>
+      <c r="C172" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E172">
         <v>0</v>
       </c>
@@ -3505,7 +3849,9 @@
       <c r="B173" s="6">
         <v>0</v>
       </c>
-      <c r="C173" s="7"/>
+      <c r="C173" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E173">
         <v>0</v>
       </c>
@@ -3517,7 +3863,9 @@
       <c r="B174" s="6">
         <v>0</v>
       </c>
-      <c r="C174" s="7"/>
+      <c r="C174" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E174">
         <v>0</v>
       </c>
@@ -3529,7 +3877,9 @@
       <c r="B175" s="6">
         <v>0</v>
       </c>
-      <c r="C175" s="7"/>
+      <c r="C175" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E175">
         <v>0</v>
       </c>
@@ -3541,7 +3891,9 @@
       <c r="B176" s="6">
         <v>0</v>
       </c>
-      <c r="C176" s="7"/>
+      <c r="C176" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E176">
         <v>0</v>
       </c>
@@ -3553,7 +3905,9 @@
       <c r="B177" s="6">
         <v>0</v>
       </c>
-      <c r="C177" s="7"/>
+      <c r="C177" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E177">
         <v>0</v>
       </c>
@@ -3565,7 +3919,9 @@
       <c r="B178" s="6">
         <v>0</v>
       </c>
-      <c r="C178" s="7"/>
+      <c r="C178" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E178">
         <v>0</v>
       </c>
@@ -3577,7 +3933,9 @@
       <c r="B179" s="6">
         <v>0</v>
       </c>
-      <c r="C179" s="7"/>
+      <c r="C179" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E179">
         <v>0</v>
       </c>
@@ -3589,7 +3947,9 @@
       <c r="B180" s="6">
         <v>0</v>
       </c>
-      <c r="C180" s="7"/>
+      <c r="C180" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E180">
         <v>0</v>
       </c>
@@ -3601,7 +3961,9 @@
       <c r="B181" s="6">
         <v>0</v>
       </c>
-      <c r="C181" s="7"/>
+      <c r="C181" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E181">
         <v>0</v>
       </c>
@@ -3613,7 +3975,9 @@
       <c r="B182" s="6">
         <v>0</v>
       </c>
-      <c r="C182" s="7"/>
+      <c r="C182" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E182">
         <v>0</v>
       </c>
@@ -3625,7 +3989,9 @@
       <c r="B183" s="6">
         <v>0</v>
       </c>
-      <c r="C183" s="7"/>
+      <c r="C183" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E183">
         <v>0</v>
       </c>
@@ -3637,7 +4003,9 @@
       <c r="B184" s="6">
         <v>0</v>
       </c>
-      <c r="C184" s="7"/>
+      <c r="C184" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E184">
         <v>0</v>
       </c>
@@ -3649,7 +4017,9 @@
       <c r="B185" s="6">
         <v>0</v>
       </c>
-      <c r="C185" s="7"/>
+      <c r="C185" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E185">
         <v>0</v>
       </c>
@@ -3661,7 +4031,9 @@
       <c r="B186" s="6">
         <v>0</v>
       </c>
-      <c r="C186" s="7"/>
+      <c r="C186" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E186">
         <v>0</v>
       </c>
@@ -3673,7 +4045,9 @@
       <c r="B187" s="6">
         <v>0</v>
       </c>
-      <c r="C187" s="7"/>
+      <c r="C187" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E187">
         <v>0</v>
       </c>
@@ -3685,7 +4059,9 @@
       <c r="B188" s="6">
         <v>0</v>
       </c>
-      <c r="C188" s="7"/>
+      <c r="C188" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E188">
         <v>0</v>
       </c>
@@ -3697,7 +4073,9 @@
       <c r="B189" s="6">
         <v>0</v>
       </c>
-      <c r="C189" s="7"/>
+      <c r="C189" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E189">
         <v>0</v>
       </c>
@@ -3709,7 +4087,9 @@
       <c r="B190" s="6">
         <v>0</v>
       </c>
-      <c r="C190" s="7"/>
+      <c r="C190" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E190">
         <v>0</v>
       </c>
@@ -3721,7 +4101,9 @@
       <c r="B191" s="6">
         <v>0</v>
       </c>
-      <c r="C191" s="7"/>
+      <c r="C191" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E191">
         <v>0</v>
       </c>
@@ -3733,7 +4115,9 @@
       <c r="B192" s="6">
         <v>0</v>
       </c>
-      <c r="C192" s="7"/>
+      <c r="C192" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E192">
         <v>0</v>
       </c>
@@ -3745,7 +4129,9 @@
       <c r="B193" s="6">
         <v>0</v>
       </c>
-      <c r="C193" s="7"/>
+      <c r="C193" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E193">
         <v>0</v>
       </c>
@@ -3757,7 +4143,9 @@
       <c r="B194" s="6">
         <v>0</v>
       </c>
-      <c r="C194" s="7"/>
+      <c r="C194" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E194">
         <v>0</v>
       </c>
@@ -3769,7 +4157,9 @@
       <c r="B195" s="6">
         <v>0</v>
       </c>
-      <c r="C195" s="7"/>
+      <c r="C195" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E195">
         <v>0</v>
       </c>
@@ -3781,7 +4171,9 @@
       <c r="B196" s="6">
         <v>0</v>
       </c>
-      <c r="C196" s="7"/>
+      <c r="C196" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E196">
         <v>0</v>
       </c>
@@ -3793,7 +4185,9 @@
       <c r="B197" s="6">
         <v>0</v>
       </c>
-      <c r="C197" s="7"/>
+      <c r="C197" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E197">
         <v>0</v>
       </c>
@@ -3805,7 +4199,9 @@
       <c r="B198" s="6">
         <v>0</v>
       </c>
-      <c r="C198" s="7"/>
+      <c r="C198" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E198">
         <v>0</v>
       </c>
@@ -3817,7 +4213,9 @@
       <c r="B199" s="6">
         <v>0</v>
       </c>
-      <c r="C199" s="7"/>
+      <c r="C199" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E199">
         <v>0</v>
       </c>
@@ -3829,7 +4227,9 @@
       <c r="B200" s="6">
         <v>0</v>
       </c>
-      <c r="C200" s="7"/>
+      <c r="C200" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E200">
         <v>0</v>
       </c>
@@ -3841,7 +4241,9 @@
       <c r="B201" s="6">
         <v>0</v>
       </c>
-      <c r="C201" s="7"/>
+      <c r="C201" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E201">
         <v>0</v>
       </c>
@@ -3853,7 +4255,9 @@
       <c r="B202" s="6">
         <v>0</v>
       </c>
-      <c r="C202" s="7"/>
+      <c r="C202" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E202">
         <v>0</v>
       </c>
@@ -3865,7 +4269,9 @@
       <c r="B203" s="6">
         <v>0</v>
       </c>
-      <c r="C203" s="7"/>
+      <c r="C203" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E203">
         <v>0</v>
       </c>
@@ -3877,7 +4283,9 @@
       <c r="B204" s="6">
         <v>0</v>
       </c>
-      <c r="C204" s="7"/>
+      <c r="C204" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E204">
         <v>0</v>
       </c>
@@ -3889,7 +4297,9 @@
       <c r="B205" s="6">
         <v>0</v>
       </c>
-      <c r="C205" s="7"/>
+      <c r="C205" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E205">
         <v>0</v>
       </c>
@@ -3901,7 +4311,9 @@
       <c r="B206" s="6">
         <v>0</v>
       </c>
-      <c r="C206" s="7"/>
+      <c r="C206" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E206">
         <v>0</v>
       </c>
@@ -3913,7 +4325,9 @@
       <c r="B207" s="6">
         <v>0</v>
       </c>
-      <c r="C207" s="7"/>
+      <c r="C207" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E207">
         <v>0</v>
       </c>
@@ -3925,7 +4339,9 @@
       <c r="B208" s="6">
         <v>0</v>
       </c>
-      <c r="C208" s="7"/>
+      <c r="C208" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E208">
         <v>0</v>
       </c>
@@ -3937,7 +4353,9 @@
       <c r="B209" s="6">
         <v>0</v>
       </c>
-      <c r="C209" s="7"/>
+      <c r="C209" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E209">
         <v>0</v>
       </c>
@@ -3949,7 +4367,9 @@
       <c r="B210" s="6">
         <v>0</v>
       </c>
-      <c r="C210" s="7"/>
+      <c r="C210" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E210">
         <v>0</v>
       </c>
@@ -3961,7 +4381,9 @@
       <c r="B211" s="6">
         <v>0</v>
       </c>
-      <c r="C211" s="7"/>
+      <c r="C211" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E211">
         <v>0</v>
       </c>
@@ -3973,7 +4395,9 @@
       <c r="B212" s="6">
         <v>0</v>
       </c>
-      <c r="C212" s="7"/>
+      <c r="C212" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E212">
         <v>0</v>
       </c>
@@ -3985,7 +4409,9 @@
       <c r="B213" s="6">
         <v>0</v>
       </c>
-      <c r="C213" s="7"/>
+      <c r="C213" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E213">
         <v>0</v>
       </c>
@@ -3997,7 +4423,9 @@
       <c r="B214" s="6">
         <v>0</v>
       </c>
-      <c r="C214" s="7"/>
+      <c r="C214" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E214">
         <v>0</v>
       </c>
@@ -4009,7 +4437,9 @@
       <c r="B215" s="6">
         <v>0</v>
       </c>
-      <c r="C215" s="7"/>
+      <c r="C215" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E215">
         <v>0</v>
       </c>
@@ -4021,7 +4451,9 @@
       <c r="B216" s="6">
         <v>0</v>
       </c>
-      <c r="C216" s="7"/>
+      <c r="C216" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E216">
         <v>0</v>
       </c>
@@ -4033,7 +4465,9 @@
       <c r="B217" s="6">
         <v>0</v>
       </c>
-      <c r="C217" s="7"/>
+      <c r="C217" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E217">
         <v>0</v>
       </c>
@@ -4045,7 +4479,9 @@
       <c r="B218" s="6">
         <v>0</v>
       </c>
-      <c r="C218" s="7"/>
+      <c r="C218" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E218">
         <v>0</v>
       </c>
@@ -4057,7 +4493,9 @@
       <c r="B219" s="6">
         <v>0</v>
       </c>
-      <c r="C219" s="7"/>
+      <c r="C219" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E219">
         <v>0</v>
       </c>
@@ -4069,7 +4507,9 @@
       <c r="B220" s="6">
         <v>0</v>
       </c>
-      <c r="C220" s="7"/>
+      <c r="C220" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E220">
         <v>0</v>
       </c>
@@ -4081,7 +4521,9 @@
       <c r="B221" s="6">
         <v>0</v>
       </c>
-      <c r="C221" s="7"/>
+      <c r="C221" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E221">
         <v>0</v>
       </c>
@@ -4093,7 +4535,9 @@
       <c r="B222" s="6">
         <v>0</v>
       </c>
-      <c r="C222" s="7"/>
+      <c r="C222" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E222">
         <v>0</v>
       </c>
@@ -4105,7 +4549,9 @@
       <c r="B223" s="6">
         <v>0</v>
       </c>
-      <c r="C223" s="7"/>
+      <c r="C223" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E223">
         <v>0</v>
       </c>
@@ -4117,7 +4563,9 @@
       <c r="B224" s="6">
         <v>0</v>
       </c>
-      <c r="C224" s="7"/>
+      <c r="C224" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E224">
         <v>0</v>
       </c>
@@ -4129,7 +4577,9 @@
       <c r="B225" s="6">
         <v>0</v>
       </c>
-      <c r="C225" s="7"/>
+      <c r="C225" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E225">
         <v>0</v>
       </c>
@@ -4141,7 +4591,9 @@
       <c r="B226" s="6">
         <v>0</v>
       </c>
-      <c r="C226" s="7"/>
+      <c r="C226" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E226">
         <v>0</v>
       </c>
@@ -4153,7 +4605,9 @@
       <c r="B227" s="6">
         <v>0</v>
       </c>
-      <c r="C227" s="7"/>
+      <c r="C227" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E227">
         <v>0</v>
       </c>
@@ -4165,7 +4619,9 @@
       <c r="B228" s="6">
         <v>0</v>
       </c>
-      <c r="C228" s="7"/>
+      <c r="C228" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E228">
         <v>0</v>
       </c>
@@ -4177,7 +4633,9 @@
       <c r="B229" s="6">
         <v>0</v>
       </c>
-      <c r="C229" s="7"/>
+      <c r="C229" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E229">
         <v>0</v>
       </c>
@@ -4189,7 +4647,9 @@
       <c r="B230" s="6">
         <v>0</v>
       </c>
-      <c r="C230" s="7"/>
+      <c r="C230" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E230">
         <v>0</v>
       </c>
@@ -4201,7 +4661,9 @@
       <c r="B231" s="6">
         <v>0</v>
       </c>
-      <c r="C231" s="7"/>
+      <c r="C231" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E231">
         <v>0</v>
       </c>
@@ -4213,7 +4675,9 @@
       <c r="B232" s="6">
         <v>0</v>
       </c>
-      <c r="C232" s="7"/>
+      <c r="C232" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E232">
         <v>0</v>
       </c>
@@ -4225,7 +4689,9 @@
       <c r="B233" s="6">
         <v>0</v>
       </c>
-      <c r="C233" s="7"/>
+      <c r="C233" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E233">
         <v>0</v>
       </c>
@@ -4237,7 +4703,9 @@
       <c r="B234" s="6">
         <v>0</v>
       </c>
-      <c r="C234" s="7"/>
+      <c r="C234" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E234">
         <v>0</v>
       </c>
@@ -4249,7 +4717,9 @@
       <c r="B235" s="6">
         <v>0</v>
       </c>
-      <c r="C235" s="7"/>
+      <c r="C235" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E235">
         <v>0</v>
       </c>
@@ -4261,7 +4731,9 @@
       <c r="B236" s="6">
         <v>0</v>
       </c>
-      <c r="C236" s="7"/>
+      <c r="C236" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E236">
         <v>0</v>
       </c>
@@ -4273,7 +4745,9 @@
       <c r="B237" s="6">
         <v>0</v>
       </c>
-      <c r="C237" s="7"/>
+      <c r="C237" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E237">
         <v>0</v>
       </c>
@@ -4285,7 +4759,9 @@
       <c r="B238" s="6">
         <v>0</v>
       </c>
-      <c r="C238" s="7"/>
+      <c r="C238" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E238">
         <v>0</v>
       </c>
@@ -4297,7 +4773,9 @@
       <c r="B239" s="6">
         <v>0</v>
       </c>
-      <c r="C239" s="7"/>
+      <c r="C239" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E239">
         <v>0</v>
       </c>
@@ -4309,7 +4787,9 @@
       <c r="B240" s="6">
         <v>0</v>
       </c>
-      <c r="C240" s="7"/>
+      <c r="C240" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E240">
         <v>0</v>
       </c>
@@ -4321,7 +4801,9 @@
       <c r="B241" s="6">
         <v>0</v>
       </c>
-      <c r="C241" s="7"/>
+      <c r="C241" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E241">
         <v>0</v>
       </c>
@@ -4333,7 +4815,9 @@
       <c r="B242" s="6">
         <v>0</v>
       </c>
-      <c r="C242" s="7"/>
+      <c r="C242" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E242">
         <v>0</v>
       </c>
@@ -4345,7 +4829,9 @@
       <c r="B243" s="6">
         <v>0</v>
       </c>
-      <c r="C243" s="7"/>
+      <c r="C243" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E243">
         <v>0</v>
       </c>
@@ -4357,7 +4843,9 @@
       <c r="B244" s="6">
         <v>0</v>
       </c>
-      <c r="C244" s="7"/>
+      <c r="C244" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E244">
         <v>0</v>
       </c>
@@ -4369,7 +4857,9 @@
       <c r="B245" s="6">
         <v>0</v>
       </c>
-      <c r="C245" s="7"/>
+      <c r="C245" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E245">
         <v>0</v>
       </c>
@@ -4381,7 +4871,9 @@
       <c r="B246" s="6">
         <v>0</v>
       </c>
-      <c r="C246" s="7"/>
+      <c r="C246" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E246">
         <v>0</v>
       </c>
@@ -4393,7 +4885,9 @@
       <c r="B247" s="6">
         <v>0</v>
       </c>
-      <c r="C247" s="7"/>
+      <c r="C247" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E247">
         <v>0</v>
       </c>
@@ -4405,7 +4899,9 @@
       <c r="B248" s="6">
         <v>0</v>
       </c>
-      <c r="C248" s="7"/>
+      <c r="C248" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E248">
         <v>0</v>
       </c>
@@ -4417,7 +4913,9 @@
       <c r="B249" s="6">
         <v>0</v>
       </c>
-      <c r="C249" s="7"/>
+      <c r="C249" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E249">
         <v>0</v>
       </c>
@@ -4429,7 +4927,9 @@
       <c r="B250" s="6">
         <v>0</v>
       </c>
-      <c r="C250" s="7"/>
+      <c r="C250" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E250">
         <v>0</v>
       </c>
@@ -4441,7 +4941,9 @@
       <c r="B251" s="6">
         <v>0</v>
       </c>
-      <c r="C251" s="7"/>
+      <c r="C251" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E251">
         <v>0</v>
       </c>
@@ -4453,7 +4955,9 @@
       <c r="B252" s="6">
         <v>0</v>
       </c>
-      <c r="C252" s="7"/>
+      <c r="C252" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E252">
         <v>0</v>
       </c>
@@ -4465,7 +4969,9 @@
       <c r="B253" s="6">
         <v>0</v>
       </c>
-      <c r="C253" s="7"/>
+      <c r="C253" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E253">
         <v>0</v>
       </c>
@@ -4477,7 +4983,9 @@
       <c r="B254" s="6">
         <v>0</v>
       </c>
-      <c r="C254" s="7"/>
+      <c r="C254" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E254">
         <v>0</v>
       </c>
@@ -4489,7 +4997,9 @@
       <c r="B255" s="6">
         <v>0</v>
       </c>
-      <c r="C255" s="7"/>
+      <c r="C255" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E255">
         <v>0</v>
       </c>
@@ -4501,7 +5011,9 @@
       <c r="B256" s="6">
         <v>0</v>
       </c>
-      <c r="C256" s="7"/>
+      <c r="C256" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E256">
         <v>0</v>
       </c>
@@ -4513,7 +5025,9 @@
       <c r="B257" s="6">
         <v>0</v>
       </c>
-      <c r="C257" s="7"/>
+      <c r="C257" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E257">
         <v>0</v>
       </c>
@@ -4525,7 +5039,9 @@
       <c r="B258" s="6">
         <v>0</v>
       </c>
-      <c r="C258" s="7"/>
+      <c r="C258" s="7" t="e">
+        <v>#DIV/0!</v>
+      </c>
       <c r="E258">
         <v>0</v>
       </c>

</xml_diff>